<commit_message>
Tirar as chaves de acesso do arquivo versionado
Eu tinha gerado as chaves dentro do .xlsx e commitado num repositório
público. Chave que passa por repositório público deixa de ser chave, então
as duas que gerei estão queimadas e foram descartadas.

A célula B2 de cada aba de lances agora vem com um marcador. A chave de
verdade é digitada direto na planilha do Drive, depois do upload, e nunca
existe neste repositório. O doc e o cabeçalho do Apps Script explicam o
porquê.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/COPA_REVOADA_planilha.xlsx
+++ b/dados/COPA_REVOADA_planilha.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -95,6 +95,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="9">
@@ -178,7 +182,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -277,6 +281,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1602,9 +1608,14 @@
           <t>chave_de_acesso</t>
         </is>
       </c>
-      <c r="B2" s="37" t="inlineStr">
-        <is>
-          <t>RVD-GLM7-4P84</t>
+      <c r="B2" s="38" t="inlineStr">
+        <is>
+          <t>TROQUE-ESTA-CHAVE</t>
+        </is>
+      </c>
+      <c r="C2" s="39" t="inlineStr">
+        <is>
+          <t>&lt;- digite a sua aqui, depois de subir pro Drive</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
@@ -1689,9 +1700,14 @@
           <t>chave_de_acesso</t>
         </is>
       </c>
-      <c r="B2" s="37" t="inlineStr">
-        <is>
-          <t>RVD-G3JJ-BB2P</t>
+      <c r="B2" s="38" t="inlineStr">
+        <is>
+          <t>TROQUE-ESTA-CHAVE</t>
+        </is>
+      </c>
+      <c r="C2" s="39" t="inlineStr">
+        <is>
+          <t>&lt;- digite a sua aqui, depois de subir pro Drive</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">

</xml_diff>